<commit_message>
chore: regrava saidas e documentos
O working paper passou de doze para dezoito paginas. O HTML agora sai como
index.html, para que o GitHub Pages sirva o artigo na raiz.
</commit_message>
<xml_diff>
--- a/outputs/tables/tab-1-areas.xlsx
+++ b/outputs/tables/tab-1-areas.xlsx
@@ -413,25 +413,25 @@
         </is>
       </c>
       <c r="B2">
-        <v>20516</v>
+        <v>13871</v>
       </c>
       <c r="C2">
-        <v>0.2379118736595827</v>
+        <v>0.274601686972821</v>
       </c>
       <c r="D2">
-        <v>6209</v>
+        <v>4884</v>
       </c>
       <c r="E2">
-        <v>0.1883581614801463</v>
+        <v>0.1563077912679907</v>
       </c>
       <c r="F2">
-        <v>0.1900955351920452</v>
+        <v>0.1983274457501262</v>
       </c>
       <c r="G2">
-        <v>0.1380779548682342</v>
+        <v>0.1377389733554117</v>
       </c>
       <c r="H2">
-        <v>0.04761370016844469</v>
+        <v>0.05253578224538761</v>
       </c>
       <c r="I2">
         <v>1.5</v>
@@ -443,32 +443,32 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ciências Biológicas</t>
+          <t>Ciências Agrárias</t>
         </is>
       </c>
       <c r="B3">
-        <v>2206</v>
+        <v>7142</v>
       </c>
       <c r="C3">
-        <v>0.200362647325476</v>
+        <v>0.2278073368804256</v>
       </c>
       <c r="D3">
-        <v>537</v>
+        <v>2045</v>
       </c>
       <c r="E3">
-        <v>0.1799709724238026</v>
+        <v>0.109145880574452</v>
       </c>
       <c r="F3">
-        <v>0.3830462375339982</v>
+        <v>0.2098851862223467</v>
       </c>
       <c r="G3">
-        <v>0.1599799398194584</v>
+        <v>0.1324855833210114</v>
       </c>
       <c r="H3">
-        <v>0.06463675213675214</v>
+        <v>0.04433257551152972</v>
       </c>
       <c r="I3">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="J3">
         <v>19</v>
@@ -477,32 +477,32 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ciências Agrárias</t>
+          <t>Ciências Biológicas</t>
         </is>
       </c>
       <c r="B4">
-        <v>10368</v>
+        <v>1489</v>
       </c>
       <c r="C4">
-        <v>0.1944444444444444</v>
+        <v>0.216252518468771</v>
       </c>
       <c r="D4">
-        <v>2512</v>
+        <v>393</v>
       </c>
       <c r="E4">
-        <v>0.1394434674666391</v>
+        <v>0.147037307973665</v>
       </c>
       <c r="F4">
-        <v>0.2084297839506173</v>
+        <v>0.3861652115513768</v>
       </c>
       <c r="G4">
-        <v>0.138728323699422</v>
+        <v>0.1716738197424893</v>
       </c>
       <c r="H4">
-        <v>0.04410774410774411</v>
+        <v>0.07836990595611286</v>
       </c>
       <c r="I4">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="J4">
         <v>19</v>
@@ -515,25 +515,25 @@
         </is>
       </c>
       <c r="B5">
-        <v>21946</v>
+        <v>15148</v>
       </c>
       <c r="C5">
-        <v>0.1303654424496491</v>
+        <v>0.1443094797993134</v>
       </c>
       <c r="D5">
-        <v>3264</v>
+        <v>2472</v>
       </c>
       <c r="E5">
-        <v>0.1692442552125728</v>
+        <v>0.1284461814724834</v>
       </c>
       <c r="F5">
-        <v>0.06684589446824023</v>
+        <v>0.06535516239767626</v>
       </c>
       <c r="G5">
-        <v>0.09221691212328099</v>
+        <v>0.08763572679509632</v>
       </c>
       <c r="H5">
-        <v>0.02791957495572455</v>
+        <v>0.02884022208513264</v>
       </c>
       <c r="I5">
         <v>2.125</v>
@@ -549,28 +549,28 @@
         </is>
       </c>
       <c r="B6">
-        <v>25820</v>
+        <v>17954</v>
       </c>
       <c r="C6">
-        <v>0.1023625096824167</v>
+        <v>0.1166870892280272</v>
       </c>
       <c r="D6">
-        <v>3185</v>
+        <v>2538</v>
       </c>
       <c r="E6">
-        <v>0.2458054384659889</v>
+        <v>0.2249468892261001</v>
       </c>
       <c r="F6">
-        <v>0.5119674670797831</v>
+        <v>0.5116965578701125</v>
       </c>
       <c r="G6">
-        <v>0.445798755186722</v>
+        <v>0.4610548162617507</v>
       </c>
       <c r="H6">
-        <v>0.2889992641648271</v>
+        <v>0.3161440960640427</v>
       </c>
       <c r="I6">
-        <v>1.5</v>
+        <v>1.75</v>
       </c>
       <c r="J6">
         <v>21</v>
@@ -583,25 +583,25 @@
         </is>
       </c>
       <c r="B7">
-        <v>20490</v>
+        <v>14231</v>
       </c>
       <c r="C7">
-        <v>0.09673011224987799</v>
+        <v>0.1048415431101117</v>
       </c>
       <c r="D7">
-        <v>2585</v>
+        <v>1982</v>
       </c>
       <c r="E7">
-        <v>0.21585482330468</v>
+        <v>0.1925862471770111</v>
       </c>
       <c r="F7">
-        <v>0.3707174231332357</v>
+        <v>0.371723701777809</v>
       </c>
       <c r="G7">
-        <v>0.2948855125187246</v>
+        <v>0.3116883116883117</v>
       </c>
       <c r="H7">
-        <v>0.1634908106889164</v>
+        <v>0.183275034572521</v>
       </c>
       <c r="I7">
         <v>1.5</v>
@@ -617,28 +617,28 @@
         </is>
       </c>
       <c r="B8">
-        <v>23585</v>
+        <v>16344</v>
       </c>
       <c r="C8">
-        <v>0.0826372694509222</v>
+        <v>0.09122613803230543</v>
       </c>
       <c r="D8">
-        <v>2153</v>
+        <v>1645</v>
       </c>
       <c r="E8">
-        <v>0.1658413613036823</v>
+        <v>0.1264861294583884</v>
       </c>
       <c r="F8">
-        <v>0.4690269238923044</v>
+        <v>0.4632892804698972</v>
       </c>
       <c r="G8">
-        <v>0.1971785681463101</v>
+        <v>0.1995504174694926</v>
       </c>
       <c r="H8">
-        <v>0.1242292530071768</v>
+        <v>0.1390543422310464</v>
       </c>
       <c r="I8">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="J8">
         <v>19</v>
@@ -651,25 +651,25 @@
         </is>
       </c>
       <c r="B9">
-        <v>22167</v>
+        <v>15770</v>
       </c>
       <c r="C9">
-        <v>0.07768304236026526</v>
+        <v>0.08522511097019658</v>
       </c>
       <c r="D9">
-        <v>2090</v>
+        <v>1645</v>
       </c>
       <c r="E9">
-        <v>0.2507090464547677</v>
+        <v>0.2256246085322569</v>
       </c>
       <c r="F9">
-        <v>0.3873325213154689</v>
+        <v>0.3780596068484464</v>
       </c>
       <c r="G9">
-        <v>0.291005017327885</v>
+        <v>0.3020408163265306</v>
       </c>
       <c r="H9">
-        <v>0.1400044622936189</v>
+        <v>0.1571405827097596</v>
       </c>
       <c r="I9">
         <v>1.2</v>
@@ -685,28 +685,28 @@
         </is>
       </c>
       <c r="B10">
-        <v>5631</v>
+        <v>3854</v>
       </c>
       <c r="C10">
-        <v>0.06925945657964838</v>
+        <v>0.07576543850544888</v>
       </c>
       <c r="D10">
-        <v>433</v>
+        <v>321</v>
       </c>
       <c r="E10">
-        <v>0.2182712313221108</v>
+        <v>0.186529933481153</v>
       </c>
       <c r="F10">
-        <v>0.4237258035872847</v>
+        <v>0.4234561494551116</v>
       </c>
       <c r="G10">
-        <v>0.3499025341130604</v>
+        <v>0.353923205342237</v>
       </c>
       <c r="H10">
-        <v>0.1771636675235647</v>
+        <v>0.1925287356321839</v>
       </c>
       <c r="I10">
-        <v>1.75</v>
+        <v>2</v>
       </c>
       <c r="J10">
         <v>20</v>

</xml_diff>